<commit_message>
Data sync: 69 words · 200 phrases · 0 new images
</commit_message>
<xml_diff>
--- a/update_data_folder/Vocab_Confirmed.xlsx
+++ b/update_data_folder/Vocab_Confirmed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miaofang/Desktop/VocabWorkspace/update_data_folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7869D7D2-24C3-6F4B-ABAA-C5E16644E997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F093093-CFD1-744B-817D-1CEAD35746EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5038,7 +5038,7 @@
         <v>628</v>
       </c>
       <c r="E66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="s">
         <v>659</v>
@@ -5214,7 +5214,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L12 A13:L70" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L12 A13:L65 A67:L70 A66:D66 F66:L66" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>